<commit_message>
Data-ingestion now includes a section that makes a simple ensemble (unweighted average of all available models for a given target date). Testing and troubleshooting pipeline up to that point - still not running start to finish; nlocs error to be addressed
</commit_message>
<xml_diff>
--- a/Changes Tracking.xlsx
+++ b/Changes Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilytyszka/Desktop/Research/Reich Lab/Allocation Score/Allocation Score Manuscript/utility-eval-papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{862C1195-FA83-7746-A8C6-19FF98292B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC25659-49A1-7343-B10D-1D7FFB7AC97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="580" windowWidth="25440" windowHeight="14780" xr2:uid="{11C9D71A-4E8A-6B49-B8E8-C5CA3E3420D0}"/>
   </bookViews>
@@ -38,9 +38,246 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Files Changed</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Created new folder + fork (forked from the oldest version I could)</t>
+  </si>
+  <si>
+    <t>Goal is to start fresh</t>
+  </si>
+  <si>
+    <t>Created xlsx "Changes Tracking"</t>
+  </si>
+  <si>
+    <t>Changes Tracking.xlsx</t>
+  </si>
+  <si>
+    <t>Deleted files</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Allocation Score Diagrams</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> folder + contents, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>random_undocumented_experiments</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> folder + contents, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>images</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> folder + contents, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>figures</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> folder + contents, </t>
+    </r>
+  </si>
+  <si>
+    <t>Stripped down to any file that wasn't directly relevant</t>
+  </si>
+  <si>
+    <t>Generate an estimate of need (IAS max and min)  for each date of interest</t>
+  </si>
+  <si>
+    <t>Fix model selection code to fit exact specs (and be more explicit)</t>
+  </si>
+  <si>
+    <t>[Model selection summary]</t>
+  </si>
+  <si>
+    <t>determine-model-eligibility.R</t>
+  </si>
+  <si>
+    <t>Find way to sync up date-specific resources with the code that runs the alloscore</t>
+  </si>
+  <si>
+    <t>[New script?]</t>
+  </si>
+  <si>
+    <t>targets, run-alloscore.R</t>
+  </si>
+  <si>
+    <t>[New script]</t>
+  </si>
+  <si>
+    <t>Create ensemble of eligible models</t>
+  </si>
+  <si>
+    <t>Model selection</t>
+  </si>
+  <si>
+    <t>Need estimation</t>
+  </si>
+  <si>
+    <t>TASKS TO BE DONE</t>
+  </si>
+  <si>
+    <t>[all]</t>
+  </si>
+  <si>
+    <t>Run on cluster</t>
+  </si>
+  <si>
+    <t>Summary of output</t>
+  </si>
+  <si>
+    <t>[New Report Script]</t>
+  </si>
+  <si>
+    <t>Create a model-selection report to summarize which models + horizons were included</t>
+  </si>
+  <si>
+    <t>Create a summary report</t>
+  </si>
+  <si>
+    <t>Pairwise results via Kendall's tau</t>
+  </si>
+  <si>
+    <t>Produce + archive allocation results for each date + horizon (csv)</t>
+  </si>
+  <si>
+    <t>Produce + archive allocation graphs for each date + horizon (pdf or png)</t>
+  </si>
+  <si>
+    <t>Bump chart</t>
+  </si>
+  <si>
+    <t>Mean allocation score over whole time period VS mean WIS</t>
+  </si>
+  <si>
+    <t>Run WIS for each model + horizon; mWIS</t>
+  </si>
+  <si>
+    <t>AS vs iAS over time</t>
+  </si>
+  <si>
+    <t>AS overlaid on epi curve?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See WIP Script Model Selection.R to run this </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neaten data cleaning code </t>
+  </si>
+  <si>
+    <t>data-ingestion.R</t>
+  </si>
+  <si>
+    <t>data-ingestion.R, _targets.R</t>
+  </si>
+  <si>
+    <t>Created WIP Script Data Injestion.R and made corresponding changes to _targets.R to test. NOTE: target_end_date == date_of_interest turned off so I can check the outputs.</t>
+  </si>
+  <si>
+    <t>Neaten data injestion code</t>
+  </si>
+  <si>
+    <t>Started ensemble code</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Used simple_ensemble from hubEnsembles (thanks Thomas!); </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>nlocs error has been appearing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in model eligibility code </t>
+    </r>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="mm/dd/yyyy;@"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -48,13 +285,59 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -69,8 +352,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,9 +711,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1272330-7B84-3440-A782-55DA1D9E4D1D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="53.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="54.83203125" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="4" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="7"/>
+      <c r="B22" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="7"/>
+      <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A24" s="7"/>
+      <c r="B24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="7"/>
+      <c r="B26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="7"/>
+      <c r="B28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A29" s="7"/>
+      <c r="C29" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A30" s="7"/>
+      <c r="C30" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="7"/>
+      <c r="C31" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="7"/>
+      <c r="C32" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="7"/>
+      <c r="C33" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="7"/>
+      <c r="C34" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="7"/>
+      <c r="C35" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="7"/>
+      <c r="C36" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="7"/>
+      <c r="C37" s="10"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Pipeline now works with Ks calculated from true need (not user input). The IAS Ks range from 81%-99% of true need (centered on 90%) and will calculate 5 different constraint levels (n can be changed - 5 was just to test)
</commit_message>
<xml_diff>
--- a/Changes Tracking.xlsx
+++ b/Changes Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilytyszka/Desktop/Research/Reich Lab/Allocation Score/Allocation Score Manuscript/utility-eval-papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC25659-49A1-7343-B10D-1D7FFB7AC97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7343A09-5885-CD4A-A5A8-7BC4CFA4E839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="580" windowWidth="25440" windowHeight="14780" xr2:uid="{11C9D71A-4E8A-6B49-B8E8-C5CA3E3420D0}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14780" xr2:uid="{11C9D71A-4E8A-6B49-B8E8-C5CA3E3420D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,8 +38,28 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={57F7239E-75EF-F242-9236-F2CA86D7B455}</author>
+  </authors>
+  <commentList>
+    <comment ref="C27" authorId="0" shapeId="0" xr:uid="{57F7239E-75EF-F242-9236-F2CA86D7B455}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    1. extract true need from truth data
+2. generate max and min 
+3. generate n number of in-between steps</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="70">
   <si>
     <t>Date</t>
   </si>
@@ -267,6 +287,160 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> in model eligibility code </t>
+    </r>
+  </si>
+  <si>
+    <t>Debugged all of the data cleaning targets, as well as the non-alloscore scores</t>
+  </si>
+  <si>
+    <t>In the ensembles, forecast_date was arbitrarily assigned as the date of the last submitted forecast making up the ensemble. This can be changed - it's just needed for the scoring. All targets up to score_data3 now work.</t>
+  </si>
+  <si>
+    <t>Created WIP Run Alloscore.R. Began work with a very limited set of Ks in order to keep run time down.</t>
+  </si>
+  <si>
+    <t>Read through code</t>
+  </si>
+  <si>
+    <t>run_alloscore.R</t>
+  </si>
+  <si>
+    <t>resource-constraints.R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Made function that calculates max and min (81%-99% of true need) from truth values. Made function that creates K list from max and min for each date - this will need to be incorporated into the allocation score loop for the IAS later.  </t>
+  </si>
+  <si>
+    <t>Created new script for calculating ranges of resource constraints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finalized </t>
+  </si>
+  <si>
+    <t>renamed and tested it</t>
+  </si>
+  <si>
+    <t>run-alloscore-match-K.R</t>
+  </si>
+  <si>
+    <t>Created new script that connects the resource constraints to truth data when doing alloscore</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Made new script for alloscore where K is matched to true need - function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="9"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>run_alloscore_match_k</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  takes in the resource constraint grid as an input and, from that, filters down to the date of interest (I hope this freaking works…). This is a modified version of the run_alloscore function</t>
+    </r>
+  </si>
+  <si>
+    <t>Made duplicate versions of the other functions in the process</t>
+  </si>
+  <si>
+    <t>Test and debug the new functions</t>
+  </si>
+  <si>
+    <t>run-alloscore-match-K.R, _targets.R, data_ingestion.R</t>
+  </si>
+  <si>
+    <t>Double check that the number of submissions for each model + ref date checks out</t>
+  </si>
+  <si>
+    <t>run-alloscore-match-K.R, _targets.R, data_ingestion.R, resource-constraints.R</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="9"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">run_alloscore_one_date_match_k </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">is a revised run_alloscore_one_date. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="9"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">run_and_assemble_alloscores_match_k </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">is a revised run_and_assemble_alloscores. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Some tweaks to the names of objects (they weren't consistent). _targets.R now looks to run-alloscore-match-K.R and uses those functions. For some reason, truth_data wasn't pulling right, so I tweaked get_truth_data() to return it more explicitly. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>map() now erroring a few loops down</t>
+    </r>
+  </si>
+  <si>
+    <t>Implimenting new stuff</t>
+  </si>
+  <si>
+    <t>Double checked that multiple submissions for the same ref date (ex. Submitting twice in 1 week for the same target and horizon) isn't getting treated as 2x the counties in CA…</t>
+  </si>
+  <si>
+    <t>Figured out how to make the map() error stop for 1 week horizon (different parts were using target and reference dates respectively so they were misaligned - made it so we're only using the target_end date for everything now)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> map() now erroring a few loops down for 3 week horizon</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>…turns out the data pulls weren't giving us forecasts for the correct target_end_dates &gt;:/</t>
     </r>
   </si>
 </sst>
@@ -277,7 +451,7 @@
   <numFmts count="1">
     <numFmt numFmtId="168" formatCode="mm/dd/yyyy;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -325,6 +499,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -352,7 +545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -377,6 +570,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -392,6 +591,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Emily Tyszka" id="{906E1CAE-7E49-B240-937E-DF4BA07EA05D}" userId="S::etyszka@umass.edu::6f784af8-2a76-48ec-ba86-f29675f38c21" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -709,9 +914,19 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C27" dT="2026-05-13T19:50:35.32" personId="{906E1CAE-7E49-B240-937E-DF4BA07EA05D}" id="{57F7239E-75EF-F242-9236-F2CA86D7B455}">
+    <text>1. extract true need from truth data
+2. generate max and min 
+3. generate n number of in-between steps</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1272330-7B84-3440-A782-55DA1D9E4D1D}">
-  <dimension ref="A1:D37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1272330-7B84-3440-A782-55DA1D9E4D1D}">
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" style="2" customWidth="1"/>
@@ -815,142 +1030,274 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
+    <row r="8" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>46156</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>46164</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>46164</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+    <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B23" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C23" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="7"/>
-      <c r="B22" s="1" t="s">
+    <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="7"/>
+      <c r="B24" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C24" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="7"/>
-      <c r="B23" s="1" t="s">
+    <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="7"/>
+      <c r="B25" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C25" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="7"/>
-      <c r="B24" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
       <c r="B26" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
       <c r="B28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="7"/>
+      <c r="B30" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="7"/>
-      <c r="C29" s="9" t="s">
+    <row r="31" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A31" s="7"/>
+      <c r="C31" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A30" s="7"/>
-      <c r="C30" s="9" t="s">
+    <row r="32" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A32" s="7"/>
+      <c r="C32" s="9" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="7"/>
-      <c r="C31" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="7"/>
-      <c r="C32" s="10" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
       <c r="C33" s="10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="7"/>
       <c r="C34" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="7"/>
       <c r="C35" s="10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
       <c r="C36" s="10" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="7"/>
-      <c r="C37" s="10"/>
+      <c r="C37" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="7"/>
+      <c r="C38" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="7"/>
+      <c r="C39" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>